<commit_message>
Resolver ambiguedades de inventario Ruge con las aclaraciones de Mariano
Mantel: revertir decision del 17 ago, no se compra verde, se pide el negro
a la iglesia via administracion (tarea real de Eventos, logistica solo
corrobora). Arena, pala, chuches y bateria de la Cruz quedan confirmados.
Banderas de tribu siguen sin corroborar. Se documenta el concepto de
supervision por comision (logistica corrobora, no ejecuta los 214 items)
que Mariano Jurado transmitio. Quedan 2 puntos genuinamente pendientes que
Mariano va a corroborar el mismo (panos/linterna/martillo/maletines, y el
reto real de los platos de carton).
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Ruge_tareas_por_persona_19ago2026_FINAL_con_stock.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Ruge_tareas_por_persona_19ago2026_FINAL_con_stock.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1323" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1325" uniqueCount="346">
   <si>
     <t xml:space="preserve">Ruge — Tareas asignadas a Marco Guanuchi</t>
   </si>
@@ -192,6 +192,9 @@
     <t xml:space="preserve">MANTEL VERDE PARA MESA DE CAMISETAS</t>
   </si>
   <si>
+    <t xml:space="preserve">pedir a iglesia (negro)</t>
+  </si>
+  <si>
     <t xml:space="preserve">MESA PORTÁTIL PARA CAMISETAS</t>
   </si>
   <si>
@@ -928,6 +931,9 @@
   </si>
   <si>
     <t xml:space="preserve">BANDERAS DE TRIBU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pendiente corroborar</t>
   </si>
   <si>
     <t xml:space="preserve">BATERIA MARCA BOSH</t>
@@ -2320,9 +2326,12 @@
       <c r="I22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="K22" s="1" t="n">
+      <c r="J22" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K22" s="1" t="str">
         <f aca="false">IFERROR(MAX(0,I22-IF(J22&lt;&gt;"",J22,H22)),"revisar unidad")</f>
-        <v>1</v>
+        <v>revisar unidad</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2330,13 +2339,13 @@
         <v>40</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>51</v>
@@ -2351,28 +2360,28 @@
         <v>0</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D24" s="7"/>
       <c r="E24" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H24" s="1" t="n">
         <v>8</v>
@@ -2393,7 +2402,7 @@
         <v>40</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>15</v>
@@ -2402,7 +2411,7 @@
         <v>16</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>18</v>
@@ -2429,14 +2438,14 @@
         <v>37</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>18</v>
@@ -2460,14 +2469,14 @@
         <v>37</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D27" s="7"/>
       <c r="E27" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>18</v>
@@ -2488,15 +2497,15 @@
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>18</v>
@@ -2517,10 +2526,10 @@
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
@@ -2549,10 +2558,10 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
@@ -2566,10 +2575,10 @@
         <v>39</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J30" s="1" t="n">
         <v>0</v>
@@ -2577,10 +2586,10 @@
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
@@ -2609,10 +2618,10 @@
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
@@ -2626,7 +2635,7 @@
         <v>39</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I32" s="1" t="n">
         <v>200</v>
@@ -2641,10 +2650,10 @@
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
@@ -2658,7 +2667,7 @@
         <v>39</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I33" s="1" t="n">
         <v>100</v>
@@ -2673,10 +2682,10 @@
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
@@ -2705,10 +2714,10 @@
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
@@ -2737,10 +2746,10 @@
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
@@ -2769,10 +2778,10 @@
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
@@ -2801,10 +2810,10 @@
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
@@ -2818,7 +2827,7 @@
         <v>39</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I38" s="1" t="n">
         <v>100</v>
@@ -2833,15 +2842,15 @@
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>18</v>
@@ -2865,15 +2874,15 @@
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>18</v>
@@ -2905,7 +2914,7 @@
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -2917,17 +2926,17 @@
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
       <c r="G50" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H50" s="5" t="s">
         <v>8</v>
@@ -2935,10 +2944,10 @@
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C51" s="7"/>
       <c r="D51" s="7"/>
@@ -2946,7 +2955,7 @@
       <c r="F51" s="7"/>
       <c r="G51" s="7"/>
       <c r="H51" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3957,7 +3966,7 @@
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3977,7 +3986,7 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11"/>
       <c r="B4" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -4029,16 +4038,16 @@
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13"/>
       <c r="B6" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>24</v>
@@ -4066,16 +4075,16 @@
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13"/>
       <c r="B7" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>24</v>
@@ -4103,16 +4112,16 @@
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13"/>
       <c r="B8" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>24</v>
@@ -4140,10 +4149,10 @@
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13"/>
       <c r="B9" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>15</v>
@@ -4175,7 +4184,7 @@
         <v>40</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>15</v>
@@ -4209,10 +4218,10 @@
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13"/>
       <c r="B11" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>15</v>
@@ -4244,13 +4253,13 @@
         <v>30</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>24</v>
@@ -4278,13 +4287,13 @@
         <v>30</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>24</v>
@@ -4312,13 +4321,13 @@
         <v>30</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>24</v>
@@ -4346,16 +4355,16 @@
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13"/>
       <c r="B15" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>24</v>
@@ -4380,10 +4389,10 @@
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13"/>
       <c r="B16" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>15</v>
@@ -4415,10 +4424,10 @@
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13"/>
       <c r="B17" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>15</v>
@@ -4447,10 +4456,10 @@
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="13"/>
       <c r="B18" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>15</v>
@@ -4479,16 +4488,16 @@
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13"/>
       <c r="B19" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>51</v>
@@ -4513,10 +4522,10 @@
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13"/>
       <c r="B20" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>15</v>
@@ -4546,17 +4555,17 @@
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="13"/>
       <c r="B21" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E21" s="7"/>
       <c r="F21" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>18</v>
@@ -4581,10 +4590,10 @@
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="13"/>
       <c r="B22" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>15</v>
@@ -4617,7 +4626,7 @@
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11"/>
       <c r="B24" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -4630,17 +4639,17 @@
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12"/>
       <c r="B25" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
       <c r="H25" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>8</v>
@@ -4649,10 +4658,10 @@
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="13"/>
       <c r="B26" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
@@ -5667,7 +5676,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -5708,7 +5717,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -5761,13 +5770,13 @@
         <v>30</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>32</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>24</v>
@@ -5792,10 +5801,10 @@
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>15</v>
@@ -5808,7 +5817,7 @@
         <v>18</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>150</v>
@@ -5826,10 +5835,10 @@
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>15</v>
@@ -5842,7 +5851,7 @@
         <v>18</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>48</v>
@@ -5860,10 +5869,10 @@
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>15</v>
@@ -5876,7 +5885,7 @@
         <v>18</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>20</v>
@@ -5894,29 +5903,29 @@
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>18</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>1</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J10" s="15" t="n">
         <v>0</v>
@@ -5925,17 +5934,17 @@
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="18" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>18</v>
@@ -5944,26 +5953,26 @@
         <v>19</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I11" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E12" s="18"/>
       <c r="F12" s="7"/>
@@ -5971,23 +5980,23 @@
         <v>19</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D13" s="7"/>
       <c r="E13" s="18"/>
@@ -5996,26 +6005,26 @@
         <v>19</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J13" s="15"/>
       <c r="K13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>43</v>
@@ -6024,7 +6033,7 @@
         <v>18</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>1</v>
@@ -6042,16 +6051,16 @@
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>51</v>
@@ -6060,7 +6069,7 @@
         <v>18</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>24</v>
@@ -6078,16 +6087,16 @@
     </row>
     <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>51</v>
@@ -6096,7 +6105,7 @@
         <v>18</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>2</v>
@@ -6114,10 +6123,10 @@
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>15</v>
@@ -6130,7 +6139,7 @@
         <v>18</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>1</v>
@@ -6148,19 +6157,19 @@
     </row>
     <row r="18" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>18</v>
@@ -6182,19 +6191,19 @@
     </row>
     <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>18</v>
@@ -6206,7 +6215,7 @@
         <v>100</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J19" s="15" t="n">
         <v>100</v>
@@ -6215,17 +6224,17 @@
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D20" s="7"/>
       <c r="E20" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>18</v>
@@ -6247,17 +6256,17 @@
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D21" s="7"/>
       <c r="E21" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>18</v>
@@ -6279,17 +6288,17 @@
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>18</v>
@@ -6313,17 +6322,17 @@
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>18</v>
@@ -6345,17 +6354,17 @@
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D24" s="7"/>
       <c r="E24" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>18</v>
@@ -6377,17 +6386,17 @@
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D25" s="7"/>
       <c r="E25" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>18</v>
@@ -6409,17 +6418,17 @@
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>18</v>
@@ -6443,17 +6452,17 @@
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D27" s="7"/>
       <c r="E27" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>18</v>
@@ -6475,17 +6484,17 @@
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D28" s="7"/>
       <c r="E28" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>18</v>
@@ -6507,17 +6516,17 @@
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>18</v>
@@ -6539,17 +6548,17 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D30" s="7"/>
       <c r="E30" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>18</v>
@@ -6571,17 +6580,17 @@
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D31" s="7"/>
       <c r="E31" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>18</v>
@@ -6603,17 +6612,17 @@
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D32" s="7"/>
       <c r="E32" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>18</v>
@@ -6635,17 +6644,17 @@
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D33" s="7"/>
       <c r="E33" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>18</v>
@@ -6667,17 +6676,17 @@
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F34" s="7" t="s">
         <v>18</v>
@@ -6699,17 +6708,17 @@
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>18</v>
@@ -6731,17 +6740,17 @@
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>18</v>
@@ -6763,17 +6772,17 @@
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C37" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D37" s="7"/>
       <c r="E37" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>18</v>
@@ -6795,17 +6804,17 @@
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C38" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D38" s="7"/>
       <c r="E38" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>18</v>
@@ -6827,17 +6836,17 @@
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C39" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D39" s="7"/>
       <c r="E39" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>18</v>
@@ -6859,17 +6868,17 @@
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D40" s="7"/>
       <c r="E40" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>18</v>
@@ -6891,17 +6900,17 @@
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C41" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D41" s="7"/>
       <c r="E41" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>18</v>
@@ -6923,17 +6932,17 @@
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C42" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D42" s="7"/>
       <c r="E42" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>18</v>
@@ -6955,17 +6964,17 @@
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C43" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D43" s="7"/>
       <c r="E43" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>18</v>
@@ -6987,19 +6996,19 @@
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C44" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E44" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>18</v>
@@ -7021,19 +7030,19 @@
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C45" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E45" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>18</v>
@@ -7055,19 +7064,19 @@
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C46" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F46" s="7" t="s">
         <v>18</v>
@@ -7089,19 +7098,19 @@
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C47" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E47" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>18</v>
@@ -7123,19 +7132,19 @@
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C48" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>18</v>
@@ -7157,17 +7166,17 @@
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C49" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D49" s="7"/>
       <c r="E49" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>18</v>
@@ -7179,7 +7188,7 @@
         <v>42</v>
       </c>
       <c r="I49" s="15" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J49" s="15" t="n">
         <v>42</v>
@@ -7188,17 +7197,17 @@
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C50" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F50" s="7" t="s">
         <v>18</v>
@@ -7207,10 +7216,10 @@
         <v>19</v>
       </c>
       <c r="H50" s="15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I50" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J50" s="15" t="n">
         <v>100</v>
@@ -7219,17 +7228,17 @@
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D51" s="7"/>
       <c r="E51" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>18</v>
@@ -7238,10 +7247,10 @@
         <v>19</v>
       </c>
       <c r="H51" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I51" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J51" s="15" t="n">
         <v>86</v>
@@ -7250,17 +7259,17 @@
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C52" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D52" s="7"/>
       <c r="E52" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F52" s="7" t="s">
         <v>18</v>
@@ -7269,10 +7278,10 @@
         <v>19</v>
       </c>
       <c r="H52" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I52" s="15" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J52" s="15" t="n">
         <v>90</v>
@@ -7281,17 +7290,17 @@
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C53" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D53" s="7"/>
       <c r="E53" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>18</v>
@@ -7313,17 +7322,17 @@
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D54" s="7"/>
       <c r="E54" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F54" s="7" t="s">
         <v>18</v>
@@ -7335,24 +7344,24 @@
         <v>0</v>
       </c>
       <c r="I54" s="15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J54" s="15"/>
       <c r="K54" s="15"/>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D55" s="7"/>
       <c r="E55" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>18</v>
@@ -7374,17 +7383,17 @@
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D56" s="7"/>
       <c r="E56" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>18</v>
@@ -7406,17 +7415,17 @@
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D57" s="7"/>
       <c r="E57" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>18</v>
@@ -7438,17 +7447,17 @@
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D58" s="7"/>
       <c r="E58" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>18</v>
@@ -7470,17 +7479,17 @@
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D59" s="7"/>
       <c r="E59" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>18</v>
@@ -7502,17 +7511,17 @@
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D60" s="7"/>
       <c r="E60" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>18</v>
@@ -7534,17 +7543,17 @@
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D61" s="7"/>
       <c r="E61" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>18</v>
@@ -7566,17 +7575,17 @@
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D62" s="7"/>
       <c r="E62" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>18</v>
@@ -7598,17 +7607,17 @@
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D63" s="7"/>
       <c r="E63" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F63" s="7" t="s">
         <v>18</v>
@@ -7620,24 +7629,24 @@
         <v>0</v>
       </c>
       <c r="I63" s="15" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J63" s="15"/>
       <c r="K63" s="15"/>
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D64" s="7"/>
       <c r="E64" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F64" s="7" t="s">
         <v>18</v>
@@ -7659,17 +7668,17 @@
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D65" s="7"/>
       <c r="E65" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F65" s="7" t="s">
         <v>18</v>
@@ -7681,7 +7690,7 @@
         <v>0</v>
       </c>
       <c r="I65" s="15" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J65" s="15" t="n">
         <v>5</v>
@@ -7690,17 +7699,17 @@
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D66" s="7"/>
       <c r="E66" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F66" s="7" t="s">
         <v>18</v>
@@ -7722,17 +7731,17 @@
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D67" s="7"/>
       <c r="E67" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F67" s="7" t="s">
         <v>18</v>
@@ -7744,24 +7753,24 @@
         <v>0</v>
       </c>
       <c r="I67" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J67" s="15"/>
       <c r="K67" s="15"/>
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D68" s="7"/>
       <c r="E68" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F68" s="7" t="s">
         <v>18</v>
@@ -7773,24 +7782,24 @@
         <v>0</v>
       </c>
       <c r="I68" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J68" s="15"/>
       <c r="K68" s="15"/>
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D69" s="7"/>
       <c r="E69" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F69" s="7" t="s">
         <v>18</v>
@@ -7812,17 +7821,17 @@
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D70" s="7"/>
       <c r="E70" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F70" s="7" t="s">
         <v>18</v>
@@ -7834,24 +7843,24 @@
         <v>0</v>
       </c>
       <c r="I70" s="15" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J70" s="15"/>
       <c r="K70" s="15"/>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D71" s="7"/>
       <c r="E71" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F71" s="7" t="s">
         <v>18</v>
@@ -7863,24 +7872,24 @@
         <v>0</v>
       </c>
       <c r="I71" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J71" s="15"/>
       <c r="K71" s="15"/>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D72" s="7"/>
       <c r="E72" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F72" s="7" t="s">
         <v>18</v>
@@ -7892,24 +7901,24 @@
         <v>0</v>
       </c>
       <c r="I72" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J72" s="15"/>
       <c r="K72" s="15"/>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D73" s="7"/>
       <c r="E73" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F73" s="7" t="s">
         <v>18</v>
@@ -7921,24 +7930,24 @@
         <v>0</v>
       </c>
       <c r="I73" s="15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="J73" s="15"/>
       <c r="K73" s="15"/>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D74" s="7"/>
       <c r="E74" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F74" s="7" t="s">
         <v>18</v>
@@ -7950,24 +7959,24 @@
         <v>0</v>
       </c>
       <c r="I74" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J74" s="15"/>
       <c r="K74" s="15"/>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D75" s="7"/>
       <c r="E75" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F75" s="7" t="s">
         <v>18</v>
@@ -7979,24 +7988,24 @@
         <v>0</v>
       </c>
       <c r="I75" s="15" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J75" s="15"/>
       <c r="K75" s="15"/>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D76" s="7"/>
       <c r="E76" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F76" s="7" t="s">
         <v>18</v>
@@ -8008,24 +8017,24 @@
         <v>0</v>
       </c>
       <c r="I76" s="15" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J76" s="15"/>
       <c r="K76" s="15"/>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D77" s="7"/>
       <c r="E77" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F77" s="7" t="s">
         <v>18</v>
@@ -8047,17 +8056,17 @@
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D78" s="7"/>
       <c r="E78" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F78" s="7" t="s">
         <v>18</v>
@@ -8079,17 +8088,17 @@
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D79" s="7"/>
       <c r="E79" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F79" s="7" t="s">
         <v>18</v>
@@ -8111,17 +8120,17 @@
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B80" s="7" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D80" s="7"/>
       <c r="E80" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F80" s="7" t="s">
         <v>18</v>
@@ -8143,17 +8152,17 @@
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D81" s="7"/>
       <c r="E81" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F81" s="7" t="s">
         <v>18</v>
@@ -8165,24 +8174,24 @@
         <v>0</v>
       </c>
       <c r="I81" s="15" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J81" s="15"/>
       <c r="K81" s="15"/>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D82" s="7"/>
       <c r="E82" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F82" s="7" t="s">
         <v>18</v>
@@ -8194,24 +8203,24 @@
         <v>0</v>
       </c>
       <c r="I82" s="15" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J82" s="15"/>
       <c r="K82" s="15"/>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D83" s="7"/>
       <c r="E83" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F83" s="7" t="s">
         <v>18</v>
@@ -8223,24 +8232,24 @@
         <v>0</v>
       </c>
       <c r="I83" s="15" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J83" s="15"/>
       <c r="K83" s="15"/>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D84" s="7"/>
       <c r="E84" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F84" s="7" t="s">
         <v>18</v>
@@ -8262,17 +8271,17 @@
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D85" s="7"/>
       <c r="E85" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F85" s="7" t="s">
         <v>18</v>
@@ -8284,24 +8293,24 @@
         <v>0</v>
       </c>
       <c r="I85" s="15" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J85" s="15"/>
       <c r="K85" s="15"/>
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D86" s="7"/>
       <c r="E86" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F86" s="7" t="s">
         <v>18</v>
@@ -8323,17 +8332,17 @@
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D87" s="7"/>
       <c r="E87" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F87" s="7" t="s">
         <v>18</v>
@@ -8345,24 +8354,24 @@
         <v>0</v>
       </c>
       <c r="I87" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J87" s="15"/>
       <c r="K87" s="15"/>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B88" s="7" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D88" s="7"/>
       <c r="E88" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F88" s="7" t="s">
         <v>18</v>
@@ -8374,24 +8383,24 @@
         <v>0</v>
       </c>
       <c r="I88" s="15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J88" s="15"/>
       <c r="K88" s="15"/>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D89" s="7"/>
       <c r="E89" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F89" s="7" t="s">
         <v>18</v>
@@ -8403,24 +8412,24 @@
         <v>0</v>
       </c>
       <c r="I89" s="15" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J89" s="15"/>
       <c r="K89" s="15"/>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B90" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D90" s="7"/>
       <c r="E90" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F90" s="7" t="s">
         <v>18</v>
@@ -8432,24 +8441,24 @@
         <v>0</v>
       </c>
       <c r="I90" s="15" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J90" s="15"/>
       <c r="K90" s="15"/>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B91" s="7" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D91" s="7"/>
       <c r="E91" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F91" s="7" t="s">
         <v>18</v>
@@ -8471,17 +8480,17 @@
     </row>
     <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B92" s="7" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D92" s="7"/>
       <c r="E92" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F92" s="7" t="s">
         <v>18</v>
@@ -8503,17 +8512,17 @@
     </row>
     <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B93" s="7" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D93" s="7"/>
       <c r="E93" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F93" s="7" t="s">
         <v>18</v>
@@ -8535,17 +8544,17 @@
     </row>
     <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D94" s="7"/>
       <c r="E94" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F94" s="7" t="s">
         <v>18</v>
@@ -8557,24 +8566,24 @@
         <v>0</v>
       </c>
       <c r="I94" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J94" s="15"/>
       <c r="K94" s="15"/>
     </row>
     <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B95" s="7" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D95" s="7"/>
       <c r="E95" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F95" s="7" t="s">
         <v>18</v>
@@ -8586,24 +8595,24 @@
         <v>0</v>
       </c>
       <c r="I95" s="15" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J95" s="15"/>
       <c r="K95" s="15"/>
     </row>
     <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B96" s="7" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D96" s="7"/>
       <c r="E96" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F96" s="7" t="s">
         <v>18</v>
@@ -8623,17 +8632,17 @@
     </row>
     <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B97" s="7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D97" s="7"/>
       <c r="E97" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F97" s="7" t="s">
         <v>18</v>
@@ -8645,24 +8654,24 @@
         <v>0</v>
       </c>
       <c r="I97" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J97" s="15"/>
       <c r="K97" s="15"/>
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B98" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D98" s="7"/>
       <c r="E98" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F98" s="7" t="s">
         <v>18</v>
@@ -8674,24 +8683,24 @@
         <v>0</v>
       </c>
       <c r="I98" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J98" s="15"/>
       <c r="K98" s="15"/>
     </row>
     <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B99" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D99" s="7"/>
       <c r="E99" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F99" s="7" t="s">
         <v>18</v>
@@ -8703,24 +8712,24 @@
         <v>0</v>
       </c>
       <c r="I99" s="15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="J99" s="15"/>
       <c r="K99" s="15"/>
     </row>
     <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D100" s="7"/>
       <c r="E100" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F100" s="7" t="s">
         <v>18</v>
@@ -8732,24 +8741,24 @@
         <v>0</v>
       </c>
       <c r="I100" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J100" s="15"/>
       <c r="K100" s="15"/>
     </row>
     <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B101" s="7" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D101" s="7"/>
       <c r="E101" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F101" s="7" t="s">
         <v>18</v>
@@ -8761,24 +8770,24 @@
         <v>0</v>
       </c>
       <c r="I101" s="15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="J101" s="15"/>
       <c r="K101" s="15"/>
     </row>
     <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B102" s="7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D102" s="7"/>
       <c r="E102" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F102" s="7" t="s">
         <v>18</v>
@@ -8800,17 +8809,17 @@
     </row>
     <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B103" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C103" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D103" s="7"/>
       <c r="E103" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F103" s="7" t="s">
         <v>18</v>
@@ -8832,17 +8841,17 @@
     </row>
     <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D104" s="7"/>
       <c r="E104" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F104" s="7" t="s">
         <v>18</v>
@@ -8854,24 +8863,24 @@
         <v>0</v>
       </c>
       <c r="I104" s="15" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J104" s="15"/>
       <c r="K104" s="15"/>
     </row>
     <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B105" s="7" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D105" s="7"/>
       <c r="E105" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F105" s="7" t="s">
         <v>18</v>
@@ -8883,24 +8892,24 @@
         <v>0</v>
       </c>
       <c r="I105" s="15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="J105" s="15"/>
       <c r="K105" s="15"/>
     </row>
     <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D106" s="7"/>
       <c r="E106" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F106" s="7" t="s">
         <v>18</v>
@@ -8912,24 +8921,24 @@
         <v>0</v>
       </c>
       <c r="I106" s="15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J106" s="15"/>
       <c r="K106" s="15"/>
     </row>
     <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B107" s="7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D107" s="7"/>
       <c r="E107" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F107" s="7" t="s">
         <v>18</v>
@@ -8941,7 +8950,7 @@
         <v>0</v>
       </c>
       <c r="I107" s="15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J107" s="15" t="n">
         <v>2</v>
@@ -8950,17 +8959,17 @@
     </row>
     <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B108" s="7" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D108" s="7"/>
       <c r="E108" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F108" s="7" t="s">
         <v>18</v>
@@ -8972,24 +8981,24 @@
         <v>0</v>
       </c>
       <c r="I108" s="15" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J108" s="15"/>
       <c r="K108" s="15"/>
     </row>
     <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B109" s="7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C109" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D109" s="7"/>
       <c r="E109" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F109" s="7" t="s">
         <v>18</v>
@@ -9001,24 +9010,24 @@
         <v>0</v>
       </c>
       <c r="I109" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J109" s="15"/>
       <c r="K109" s="15"/>
     </row>
     <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B110" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D110" s="7"/>
       <c r="E110" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F110" s="7" t="s">
         <v>18</v>
@@ -9030,24 +9039,24 @@
         <v>0</v>
       </c>
       <c r="I110" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J110" s="15"/>
       <c r="K110" s="15"/>
     </row>
     <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B111" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D111" s="7"/>
       <c r="E111" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F111" s="7" t="s">
         <v>18</v>
@@ -9069,17 +9078,17 @@
     </row>
     <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B112" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D112" s="7"/>
       <c r="E112" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F112" s="7" t="s">
         <v>18</v>
@@ -9101,22 +9110,22 @@
     </row>
     <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B113" s="7" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C113" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D113" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E113" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F113" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G113" s="7" t="s">
         <v>19</v>
@@ -9137,31 +9146,31 @@
     </row>
     <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B114" s="7" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C114" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D114" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E114" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F114" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G114" s="7" t="s">
         <v>19</v>
       </c>
       <c r="H114" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I114" s="15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J114" s="15" t="n">
         <v>2</v>
@@ -9170,31 +9179,31 @@
     </row>
     <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B115" s="7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C115" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D115" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E115" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F115" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G115" s="7" t="s">
         <v>19</v>
       </c>
       <c r="H115" s="15" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I115" s="15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J115" s="15" t="n">
         <v>4</v>
@@ -9203,22 +9212,22 @@
     </row>
     <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B116" s="7" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C116" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D116" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E116" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F116" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G116" s="7" t="s">
         <v>19</v>
@@ -9239,22 +9248,22 @@
     </row>
     <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B117" s="7" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C117" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D117" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E117" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F117" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G117" s="7" t="s">
         <v>19</v>
@@ -9275,22 +9284,22 @@
     </row>
     <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B118" s="7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C118" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D118" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E118" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F118" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G118" s="7" t="s">
         <v>19</v>
@@ -9311,31 +9320,31 @@
     </row>
     <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B119" s="7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C119" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D119" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E119" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F119" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G119" s="7" t="s">
         <v>19</v>
       </c>
       <c r="H119" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I119" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J119" s="15" t="n">
         <v>2</v>
@@ -9344,15 +9353,15 @@
     </row>
     <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B120" s="9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C120" s="9"/>
       <c r="D120" s="9"/>
       <c r="E120" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>18</v>
@@ -9374,10 +9383,10 @@
     </row>
     <row r="121" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B121" s="9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C121" s="9"/>
       <c r="D121" s="9"/>
@@ -9404,10 +9413,10 @@
     </row>
     <row r="122" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B122" s="9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C122" s="9"/>
       <c r="D122" s="9"/>
@@ -9436,15 +9445,15 @@
     </row>
     <row r="123" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B123" s="9" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C123" s="9"/>
       <c r="D123" s="9"/>
       <c r="E123" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>18</v>
@@ -9468,15 +9477,15 @@
     </row>
     <row r="124" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B124" s="9" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C124" s="9"/>
       <c r="D124" s="9"/>
       <c r="E124" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>18</v>
@@ -9500,10 +9509,10 @@
     </row>
     <row r="125" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B125" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C125" s="9"/>
       <c r="D125" s="9"/>
@@ -9532,15 +9541,15 @@
     </row>
     <row r="126" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B126" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C126" s="9"/>
       <c r="D126" s="9"/>
       <c r="E126" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>18</v>
@@ -9564,10 +9573,10 @@
     </row>
     <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B127" s="9" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C127" s="9"/>
       <c r="D127" s="9"/>
@@ -9575,7 +9584,7 @@
         <v>51</v>
       </c>
       <c r="F127" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G127" s="20" t="n">
         <v>46267</v>
@@ -9596,10 +9605,10 @@
     </row>
     <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B128" s="9" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C128" s="9"/>
       <c r="D128" s="9"/>
@@ -9607,7 +9616,7 @@
         <v>51</v>
       </c>
       <c r="F128" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G128" s="20" t="n">
         <v>46267</v>
@@ -9628,10 +9637,10 @@
     </row>
     <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B129" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C129" s="9"/>
       <c r="D129" s="9"/>
@@ -9639,7 +9648,7 @@
         <v>51</v>
       </c>
       <c r="F129" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G129" s="20" t="n">
         <v>46267</v>
@@ -9650,18 +9659,20 @@
       <c r="I129" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="J129" s="15"/>
-      <c r="K129" s="15" t="n">
+      <c r="J129" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="K129" s="15" t="str">
         <f aca="false">IFERROR(MAX(0,I129-IF(J129&lt;&gt;"",J129,H129)),"revisar unidad")</f>
-        <v>0</v>
+        <v>revisar unidad</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B130" s="9" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C130" s="9"/>
       <c r="D130" s="9"/>
@@ -9669,7 +9680,7 @@
         <v>51</v>
       </c>
       <c r="F130" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G130" s="20" t="n">
         <v>46267</v>
@@ -9678,19 +9689,19 @@
         <v>1</v>
       </c>
       <c r="I130" s="15" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="J130" s="15" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="K130" s="15"/>
     </row>
     <row r="131" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B131" s="9" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C131" s="9"/>
       <c r="D131" s="9"/>
@@ -9698,7 +9709,7 @@
         <v>51</v>
       </c>
       <c r="F131" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G131" s="20" t="n">
         <v>46267</v>
@@ -9719,10 +9730,10 @@
     </row>
     <row r="132" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B132" s="9" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C132" s="9"/>
       <c r="D132" s="9"/>
@@ -9730,7 +9741,7 @@
         <v>51</v>
       </c>
       <c r="F132" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G132" s="20" t="n">
         <v>46267</v>
@@ -9751,10 +9762,10 @@
     </row>
     <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B133" s="9" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C133" s="9"/>
       <c r="D133" s="9"/>
@@ -9762,7 +9773,7 @@
         <v>51</v>
       </c>
       <c r="F133" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G133" s="20" t="n">
         <v>46267</v>
@@ -9781,10 +9792,10 @@
     </row>
     <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B134" s="9" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C134" s="9"/>
       <c r="D134" s="9"/>
@@ -9792,7 +9803,7 @@
         <v>51</v>
       </c>
       <c r="F134" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G134" s="20" t="n">
         <v>46267</v>
@@ -9813,10 +9824,10 @@
     </row>
     <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B135" s="9" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C135" s="9"/>
       <c r="D135" s="9"/>
@@ -9824,7 +9835,7 @@
         <v>51</v>
       </c>
       <c r="F135" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G135" s="20" t="n">
         <v>46267</v>
@@ -9843,10 +9854,10 @@
     </row>
     <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B136" s="9" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C136" s="9"/>
       <c r="D136" s="9"/>
@@ -9854,7 +9865,7 @@
         <v>51</v>
       </c>
       <c r="F136" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G136" s="20" t="n">
         <v>46267</v>
@@ -9875,10 +9886,10 @@
     </row>
     <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B137" s="9" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C137" s="9"/>
       <c r="D137" s="9"/>
@@ -9886,7 +9897,7 @@
         <v>51</v>
       </c>
       <c r="F137" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G137" s="20" t="n">
         <v>46267</v>
@@ -9907,10 +9918,10 @@
     </row>
     <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B138" s="9" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C138" s="9"/>
       <c r="D138" s="9"/>
@@ -9918,16 +9929,16 @@
         <v>51</v>
       </c>
       <c r="F138" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G138" s="20" t="n">
         <v>46267</v>
       </c>
       <c r="H138" s="15" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="I138" s="15" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J138" s="15" t="n">
         <v>3</v>
@@ -9936,10 +9947,10 @@
     </row>
     <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B139" s="9" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C139" s="9"/>
       <c r="D139" s="9"/>
@@ -9947,7 +9958,7 @@
         <v>51</v>
       </c>
       <c r="F139" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G139" s="20" t="n">
         <v>46267</v>
@@ -9966,10 +9977,10 @@
     </row>
     <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B140" s="9" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C140" s="9"/>
       <c r="D140" s="9"/>
@@ -9977,7 +9988,7 @@
         <v>51</v>
       </c>
       <c r="F140" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G140" s="20" t="n">
         <v>46267</v>
@@ -9998,10 +10009,10 @@
     </row>
     <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B141" s="9" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C141" s="9"/>
       <c r="D141" s="9"/>
@@ -10009,7 +10020,7 @@
         <v>51</v>
       </c>
       <c r="F141" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G141" s="20" t="n">
         <v>46267</v>
@@ -10028,10 +10039,10 @@
     </row>
     <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B142" s="9" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C142" s="9"/>
       <c r="D142" s="9"/>
@@ -10039,7 +10050,7 @@
         <v>51</v>
       </c>
       <c r="F142" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G142" s="20" t="n">
         <v>46267</v>
@@ -10060,10 +10071,10 @@
     </row>
     <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B143" s="9" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C143" s="9"/>
       <c r="D143" s="9"/>
@@ -10071,7 +10082,7 @@
         <v>51</v>
       </c>
       <c r="F143" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G143" s="20" t="n">
         <v>46267</v>
@@ -10092,10 +10103,10 @@
     </row>
     <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B144" s="9" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C144" s="9"/>
       <c r="D144" s="9"/>
@@ -10103,7 +10114,7 @@
         <v>51</v>
       </c>
       <c r="F144" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G144" s="20" t="n">
         <v>46267</v>
@@ -10124,10 +10135,10 @@
     </row>
     <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B145" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C145" s="9"/>
       <c r="D145" s="9"/>
@@ -10135,7 +10146,7 @@
         <v>51</v>
       </c>
       <c r="F145" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G145" s="20" t="n">
         <v>46267</v>
@@ -10156,10 +10167,10 @@
     </row>
     <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B146" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C146" s="9"/>
       <c r="D146" s="9"/>
@@ -10167,7 +10178,7 @@
         <v>51</v>
       </c>
       <c r="F146" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G146" s="20" t="n">
         <v>46267</v>
@@ -10176,7 +10187,7 @@
         <v>5</v>
       </c>
       <c r="I146" s="15" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J146" s="15" t="n">
         <v>0</v>
@@ -10185,10 +10196,10 @@
     </row>
     <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B147" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C147" s="9"/>
       <c r="D147" s="9"/>
@@ -10196,7 +10207,7 @@
         <v>51</v>
       </c>
       <c r="F147" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G147" s="20" t="n">
         <v>46267</v>
@@ -10217,18 +10228,18 @@
     </row>
     <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B148" s="9" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C148" s="9"/>
       <c r="D148" s="9"/>
       <c r="E148" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F148" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G148" s="20" t="n">
         <v>46267</v>
@@ -10249,18 +10260,18 @@
     </row>
     <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B149" s="9" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C149" s="9"/>
       <c r="D149" s="9"/>
       <c r="E149" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F149" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G149" s="20" t="n">
         <v>46267</v>
@@ -10281,18 +10292,18 @@
     </row>
     <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B150" s="9" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C150" s="9"/>
       <c r="D150" s="9"/>
       <c r="E150" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F150" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G150" s="20" t="n">
         <v>46267</v>
@@ -10301,17 +10312,17 @@
         <v>6</v>
       </c>
       <c r="I150" s="15" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="J150" s="15"/>
       <c r="K150" s="15"/>
     </row>
     <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B151" s="9" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C151" s="9"/>
       <c r="D151" s="9"/>
@@ -10319,7 +10330,7 @@
         <v>43</v>
       </c>
       <c r="F151" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G151" s="20" t="n">
         <v>46267</v>
@@ -10340,10 +10351,10 @@
     </row>
     <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B152" s="9" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C152" s="9"/>
       <c r="D152" s="9"/>
@@ -10351,7 +10362,7 @@
         <v>43</v>
       </c>
       <c r="F152" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G152" s="20" t="n">
         <v>46267</v>
@@ -10372,10 +10383,10 @@
     </row>
     <row r="153" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B153" s="9" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C153" s="9"/>
       <c r="D153" s="9"/>
@@ -10402,10 +10413,10 @@
     </row>
     <row r="154" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B154" s="9" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C154" s="9"/>
       <c r="D154" s="9"/>
@@ -10434,10 +10445,10 @@
     </row>
     <row r="155" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B155" s="9" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C155" s="9"/>
       <c r="D155" s="9"/>
@@ -11346,12 +11357,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -11363,7 +11374,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -11375,17 +11386,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>8</v>
@@ -11393,10 +11404,10 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -11404,54 +11415,54 @@
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
       <c r="G8" s="7" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H9" s="7"/>
     </row>

</xml_diff>